<commit_message>
Mejora en logica de guaraddo de informcion, valdiaciones especiales en microservicio
</commit_message>
<xml_diff>
--- a/backend/src/assets/templates/Consolidado_PostNomina_Cierre.xlsx
+++ b/backend/src/assets/templates/Consolidado_PostNomina_Cierre.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\camig\MIENTRAS TANTO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3e335d3f3ef462b1/Documentos/COSAS U/SEMESTRE 9/PRACTICAS/PROYECTO/BACKEND/PRACTICAS-BACK/backend/src/assets/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1051946A-5916-4240-A71C-3BE6620450F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{1051946A-5916-4240-A71C-3BE6620450F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{767EC0B4-D88E-4DDD-96E4-550CD4DA2279}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{9DDDBFE6-9518-4E38-A31B-9C6D0A783B78}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9DDDBFE6-9518-4E38-A31B-9C6D0A783B78}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>ID</t>
   </si>
@@ -133,6 +133,9 @@
   </si>
   <si>
     <t>ESPACIO EXCLUSIVO VALIDACIÓN POST NÓMINA</t>
+  </si>
+  <si>
+    <t>DIAS A TOMAR</t>
   </si>
 </sst>
 </file>
@@ -286,7 +289,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -309,6 +312,10 @@
     <xf numFmtId="164" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
     </xf>
     <xf numFmtId="17" fontId="4" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -720,40 +727,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E82EB22B-A659-4EC6-89D0-8DED0AABBA86}">
-  <dimension ref="A2:AB6"/>
+  <dimension ref="A2:AC6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="1:28" ht="3" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:28" ht="1.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K5" s="7" t="s">
+    <row r="2" spans="1:29" ht="3" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:29" ht="1.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:29" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K5" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="L5" s="8"/>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="8"/>
-      <c r="P5" s="8"/>
-      <c r="Q5" s="8" t="s">
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="9"/>
+      <c r="P5" s="9"/>
+      <c r="Q5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="R5" s="8"/>
-      <c r="S5" s="8"/>
-      <c r="T5" s="9"/>
-      <c r="U5" s="8" t="s">
+      <c r="R5" s="9"/>
+      <c r="S5" s="9"/>
+      <c r="T5" s="10"/>
+      <c r="U5" s="7"/>
+      <c r="V5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V5" s="8"/>
-      <c r="W5" s="10" t="s">
+      <c r="W5" s="9"/>
+      <c r="X5" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="X5" s="10"/>
-      <c r="Y5" s="10"/>
-      <c r="Z5" s="10"/>
-      <c r="AA5" s="10"/>
-      <c r="AB5" s="10"/>
+      <c r="Y5" s="11"/>
+      <c r="Z5" s="11"/>
+      <c r="AA5" s="11"/>
+      <c r="AB5" s="11"/>
+      <c r="AC5" s="11"/>
     </row>
-    <row r="6" spans="1:28" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:29" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -815,27 +823,30 @@
         <v>19</v>
       </c>
       <c r="U6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="V6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="V6" s="3" t="s">
+      <c r="W6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="W6" s="4" t="s">
+      <c r="X6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="X6" s="5" t="s">
+      <c r="Y6" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="Y6" s="2" t="s">
+      <c r="Z6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z6" s="6" t="s">
+      <c r="AA6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="AA6" s="2" t="s">
+      <c r="AB6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AB6" s="2" t="s">
+      <c r="AC6" s="2" t="s">
         <v>27</v>
       </c>
     </row>
@@ -843,8 +854,8 @@
   <mergeCells count="4">
     <mergeCell ref="K5:P5"/>
     <mergeCell ref="Q5:T5"/>
-    <mergeCell ref="U5:V5"/>
-    <mergeCell ref="W5:AB5"/>
+    <mergeCell ref="V5:W5"/>
+    <mergeCell ref="X5:AC5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>